<commit_message>
ajustes a 2 líneas de investigación
</commit_message>
<xml_diff>
--- a/mad-map-data-v2.xlsx
+++ b/mad-map-data-v2.xlsx
@@ -642,10 +642,11 @@
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>Régimen sin áreas-MAD: Líneas troncales sostenidas por Laboratorios + sublíneas + temas.</t>
-        </is>
-      </c>
-    </row>
+          <t>Régimen de dos líneas de investigación (septiembre 2026), cada una con polo teórico y polo proyectual, sostenidas por Laboratorios + sublíneas + temas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="16" customHeight="1" s="24">
       <c r="A4" s="26" t="inlineStr">
         <is>
@@ -656,7 +657,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Línea (4 troncales)</t>
+          <t>Línea (2)</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -749,6 +750,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="16" customHeight="1" s="24">
       <c r="A14" s="26" t="inlineStr">
         <is>
@@ -859,6 +861,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -879,7 +882,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
     </row>
@@ -891,19 +894,19 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1" s="24">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Aconcagua Fablab</t>
+          <t>Patrimonio moderno</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
     </row>
@@ -915,7 +918,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
     </row>
@@ -927,21 +930,13 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1" s="24">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Patrimonio moderno</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
-        </is>
-      </c>
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2067,6 +2062,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -2087,12 +2083,12 @@
     <row r="5" ht="60" customHeight="1" s="24">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Investigación proyectual</t>
+          <t>Historiografía</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -2104,7 +2100,7 @@
     <row r="6" ht="60" customHeight="1" s="24">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -2114,19 +2110,19 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>presente</t>
+          <t>predominante</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1" s="24">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Teoría crítica</t>
+          <t>Investigación proyectual</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -2138,29 +2134,29 @@
     <row r="8" ht="60" customHeight="1" s="24">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Investigación proyectual</t>
+          <t>Teoría crítica</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>presente</t>
+          <t>predominante</t>
         </is>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1" s="24">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Historiografía</t>
+          <t>Investigación proyectual</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -2172,36 +2168,24 @@
     <row r="10" ht="60" customHeight="1" s="24">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Teoría crítica</t>
+          <t>Historiografía</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>predominante</t>
+          <t>presente</t>
         </is>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1" s="24">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Investigación proyectual</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>predominante</t>
-        </is>
-      </c>
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2788,6 +2772,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -2816,7 +2801,7 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>El doctorado forma investigadores para quienes la obra es origen y prueba de la tesis. Esa obra, sea edificada, fabricada, escrita o dibujada, vale como argumento por sí misma, y el discurso doctoral se construye para hacerla legible y discutible. La pregunta que esa obra está llamada a argumentar es la que el programa hace suya: cómo reinventar el habitar humano. Las cuatro líneas del doctorado aportan los principios que esa pregunta convoca: la inclusión y la autonomía como condiciones de quien habita, las ecologías del territorio como condiciones de dónde, la herencia disciplinar de la e[ad] y la teoría del proyecto como condiciones desde dónde se piensa, y el oficio y los medios técnicos como condiciones con qué se hace. Doctorarse aquí es haber producido una obra capaz de sostener esos principios al ponerse a prueba y, en su mejor versión, capaz de reformularlos.</t>
+          <t>El doctorado forma investigadores para quienes la obra es origen y prueba de la tesis. Esa obra, sea edificada, fabricada, escrita o dibujada, vale como argumento por sí misma, y el discurso doctoral se construye para hacerla legible y discutible. La pregunta que esa obra está llamada a argumentar es la que el programa hace suya: cómo reinventar el habitar humano, y la responde desde el habitar poético que funda a la Escuela. Las dos líneas del doctorado investigan ese habitar en arquitectura y en diseño: una investiga acerca del proyecto, su formación, su oficio y su teoría; la otra investiga a través del proyecto, sobre la ciudad, el territorio y sus ecologías. Cada línea lleva dentro su contraparte, teórica o proyectual. Doctorarse aquí es haber producido una obra capaz de sostener esos principios al ponerse a prueba y, en su mejor versión, capaz de reformularlos.</t>
         </is>
       </c>
     </row>
@@ -5149,17 +5134,18 @@
     <row r="1" ht="18" customHeight="1" s="24">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>01 · Líneas troncales (4 a definir — BORRADOR)</t>
+          <t>01 · Líneas de investigación (2, propuesta septiembre 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>Cada Sublínea pertenece a una Línea. Los Laboratorios pueden sostener una o varias Líneas. Borrador derivado de la hipótesis de compactación.</t>
-        </is>
-      </c>
-    </row>
+          <t>Cada Sublínea pertenece a una Línea y a un polo (teórico | proyectual). Los Laboratorios pueden sostener una o varias Líneas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -5190,17 +5176,17 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Investigación sobre las condiciones de quien habita: accesibilidad e inclusión, codiseño, comunicación aumentativa y alternativa, diseño de interacción y servicios, sistemas inteligentes orientados a la diversidad funcional, la autonomía y la democracia.</t>
+          <t>Investigación acerca del proyecto de arquitectura y de diseño: cómo se forma, cómo se ejerce como oficio y desde qué teoría e historia se piensa. Acervo de la e[ad] y Ciudad Abierta, historia y crítica de la arquitectura y del diseño, teoría del proyecto y sus categorías (hospitalidad, vacío, palabra poética), espacios y medios del aprendizaje, métodos de diseño, interacción, accesibilidad, fabricación y tecnologías. Forma a quienes enseñarán arquitectura y diseño. Polo teórico e histórico y polo proyectual.</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>consolidada</t>
+          <t>propuesta 2026</t>
         </is>
       </c>
     </row>
@@ -5212,63 +5198,31 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Investigación sobre las condiciones de dónde se habita: ciudad, urbanización, ecología política, patrimonio territorial, borde costero, infraestructura urbana, vulnerabilidad y adaptación, prácticas urbanas colectivas y reuso del territorio.</t>
+          <t>Investigación a través del proyecto de arquitectura y de diseño sobre la ciudad, el territorio y sus ecologías: urbanización, ecología política, vivienda, patrimonio, borde costero, infraestructura y equipamiento, prácticas colectivas, urbanismo afectivo, diseño social y territorial. Polo teórico (teoría urbana, ecología política, vivienda) y polo proyectual (intervención, equipamiento, investigación-acción, creación de obra).</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>consolidada</t>
+          <t>propuesta 2026</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" s="24">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>LIN-03</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Investigación sobre las condiciones desde dónde se piensa: acervo histórico de la e[ad] y Ciudad Abierta, historia y crítica de la arquitectura moderna, teoría del proyecto, conceptos disciplinares como hospitalidad y vacío arquitectónico.</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>consolidada</t>
-        </is>
-      </c>
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1" s="24">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>LIN-04</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Investigación sobre las condiciones con qué se hace y cómo se transmite: métodos de diseño, oficio, saberes técnicos, fabricación digital y transferencia tecnológica, espacios educativos y pedagogía del proyecto.</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>consolidada</t>
-        </is>
-      </c>
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5285,7 +5239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="24" min="1" max="1"/>
@@ -5305,10 +5259,11 @@
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>Cada sublínea pertenece a UNA línea troncal. La asignación linea_id es BORRADOR — revisar caso por caso.</t>
-        </is>
-      </c>
-    </row>
+          <t>Cada sublínea pertenece a UNA línea y a UN polo. Reasignación de septiembre 2026 (dos líneas); revisar caso por caso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -5335,6 +5290,11 @@
           <t>notas</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>polo</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="60" customHeight="1" s="24">
       <c r="A5" s="8" t="inlineStr">
@@ -5349,7 +5309,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -5358,6 +5318,11 @@
         </is>
       </c>
       <c r="E5" s="8" t="n"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="60" customHeight="1" s="24">
       <c r="A6" s="8" t="inlineStr">
@@ -5372,7 +5337,7 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -5381,6 +5346,11 @@
         </is>
       </c>
       <c r="E6" s="8" t="n"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1" s="24">
       <c r="A7" s="8" t="inlineStr">
@@ -5395,7 +5365,7 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -5404,6 +5374,11 @@
         </is>
       </c>
       <c r="E7" s="8" t="n"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>teórico</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="60" customHeight="1" s="24">
       <c r="A8" s="8" t="inlineStr">
@@ -5418,7 +5393,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -5427,6 +5402,11 @@
         </is>
       </c>
       <c r="E8" s="8" t="n"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="60" customHeight="1" s="24">
       <c r="A9" s="8" t="inlineStr">
@@ -5441,7 +5421,7 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -5450,6 +5430,11 @@
         </is>
       </c>
       <c r="E9" s="8" t="n"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="75" customHeight="1" s="24">
       <c r="A10" s="8" t="inlineStr">
@@ -5464,7 +5449,7 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -5475,6 +5460,11 @@
       <c r="E10" s="8" t="inlineStr">
         <is>
           <t>migró a LIN-04 (aprendizaje proyectual)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -5491,7 +5481,7 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -5500,6 +5490,11 @@
         </is>
       </c>
       <c r="E11" s="8" t="n"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="75" customHeight="1" s="24">
       <c r="A12" s="8" t="inlineStr">
@@ -5514,7 +5509,7 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -5523,6 +5518,11 @@
         </is>
       </c>
       <c r="E12" s="8" t="n"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>teórico</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="75" customHeight="1" s="24">
       <c r="A13" s="8" t="inlineStr">
@@ -5537,7 +5537,7 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -5548,6 +5548,11 @@
       <c r="E13" s="8" t="inlineStr">
         <is>
           <t>migró a LIN-04</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -5564,7 +5569,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -5573,6 +5578,11 @@
         </is>
       </c>
       <c r="E14" s="8" t="n"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="60" customHeight="1" s="24">
       <c r="A15" s="8" t="inlineStr">
@@ -5587,7 +5597,7 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -5596,6 +5606,11 @@
         </is>
       </c>
       <c r="E15" s="8" t="n"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="75" customHeight="1" s="24">
       <c r="A16" s="8" t="inlineStr">
@@ -5610,7 +5625,7 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -5619,6 +5634,11 @@
         </is>
       </c>
       <c r="E16" s="8" t="n"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>teórico</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="75" customHeight="1" s="24">
       <c r="A17" s="8" t="inlineStr">
@@ -5633,7 +5653,7 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -5642,6 +5662,11 @@
         </is>
       </c>
       <c r="E17" s="8" t="n"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>teórico</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="75" customHeight="1" s="24">
       <c r="A18" s="8" t="inlineStr">
@@ -5656,7 +5681,7 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -5667,6 +5692,11 @@
       <c r="E18" s="8" t="inlineStr">
         <is>
           <t>migró a LIN-04</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5713,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -5694,6 +5724,11 @@
       <c r="E19" s="8" t="inlineStr">
         <is>
           <t>migró a LIN-04</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -5710,7 +5745,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -5721,6 +5756,11 @@
       <c r="E20" s="8" t="inlineStr">
         <is>
           <t>migró a LIN-04</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -5737,7 +5777,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -5746,6 +5786,11 @@
         </is>
       </c>
       <c r="E21" s="8" t="n"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="60" customHeight="1" s="24">
       <c r="A22" s="8" t="inlineStr">
@@ -5760,7 +5805,7 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -5769,6 +5814,11 @@
         </is>
       </c>
       <c r="E22" s="8" t="n"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="75" customHeight="1" s="24">
       <c r="A23" s="8" t="inlineStr">
@@ -5783,7 +5833,7 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -5794,6 +5844,11 @@
       <c r="E23" s="8" t="inlineStr">
         <is>
           <t>migró a LIN-04</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -5810,7 +5865,7 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -5819,6 +5874,11 @@
         </is>
       </c>
       <c r="E24" s="8" t="n"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="60" customHeight="1" s="24">
       <c r="A25" s="8" t="inlineStr">
@@ -5833,7 +5893,7 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
@@ -5844,6 +5904,11 @@
       <c r="E25" s="8" t="inlineStr">
         <is>
           <t>podría leerse en LIN-01 según énfasis</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>teórico</t>
         </is>
       </c>
     </row>
@@ -5860,7 +5925,7 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -5871,6 +5936,11 @@
       <c r="E26" s="8" t="inlineStr">
         <is>
           <t>transversal — colocar donde tenga más respaldo</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -5887,7 +5957,7 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -5898,6 +5968,11 @@
       <c r="E27" s="8" t="inlineStr">
         <is>
           <t>migró a LIN-04</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -5914,7 +5989,7 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -5925,6 +6000,11 @@
       <c r="E28" s="8" t="inlineStr">
         <is>
           <t>migró a LIN-04</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -5941,7 +6021,7 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -5950,6 +6030,11 @@
         </is>
       </c>
       <c r="E29" s="8" t="n"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="75" customHeight="1" s="24">
       <c r="A30" s="8" t="inlineStr">
@@ -5964,7 +6049,7 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -5973,6 +6058,11 @@
         </is>
       </c>
       <c r="E30" s="8" t="n"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>teórico</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1" s="24">
       <c r="A31" s="8" t="inlineStr">
@@ -5987,7 +6077,7 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -5996,6 +6086,11 @@
         </is>
       </c>
       <c r="E31" s="8" t="n"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="60" customHeight="1" s="24">
       <c r="A32" s="8" t="inlineStr">
@@ -6010,7 +6105,7 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -6019,6 +6114,11 @@
         </is>
       </c>
       <c r="E32" s="8" t="n"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="60" customHeight="1" s="24">
       <c r="A33" s="8" t="inlineStr">
@@ -6033,7 +6133,7 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -6042,6 +6142,11 @@
         </is>
       </c>
       <c r="E33" s="8" t="n"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>teórico</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="60" customHeight="1" s="24">
       <c r="A34" s="8" t="inlineStr">
@@ -6056,7 +6161,7 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -6065,6 +6170,11 @@
         </is>
       </c>
       <c r="E34" s="8" t="n"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>proyectual</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="60" customHeight="1" s="24">
       <c r="A35" s="8" t="inlineStr">
@@ -6079,7 +6189,7 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -6090,6 +6200,11 @@
       <c r="E35" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>teórico</t>
         </is>
       </c>
     </row>
@@ -6106,7 +6221,7 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -6117,6 +6232,11 @@
       <c r="E36" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>teórico</t>
         </is>
       </c>
     </row>
@@ -6133,7 +6253,7 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
@@ -6144,6 +6264,11 @@
       <c r="E37" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6285,7 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
@@ -6171,6 +6296,11 @@
       <c r="E38" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6187,7 +6317,7 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -6198,6 +6328,11 @@
       <c r="E39" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6214,7 +6349,7 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -6225,6 +6360,11 @@
       <c r="E40" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6381,7 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
@@ -6252,6 +6392,11 @@
       <c r="E41" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6413,7 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
@@ -6279,6 +6424,11 @@
       <c r="E42" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6445,7 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
@@ -6306,6 +6456,11 @@
       <c r="E43" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>teórico</t>
         </is>
       </c>
     </row>
@@ -6322,7 +6477,7 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
@@ -6333,6 +6488,11 @@
       <c r="E44" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6349,7 +6509,7 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
@@ -6360,6 +6520,11 @@
       <c r="E45" s="8" t="inlineStr">
         <is>
           <t>nueva — núcleo Jeldes</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6541,7 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
@@ -6387,6 +6552,11 @@
       <c r="E46" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6573,7 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
@@ -6414,6 +6584,11 @@
       <c r="E47" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6430,7 +6605,7 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
@@ -6441,6 +6616,11 @@
       <c r="E48" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6457,7 +6637,7 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Habitar, infraestructura y ecologías territoriales</t>
+          <t>Proyecto, ciudad y ecologías del territorio</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -6468,6 +6648,11 @@
       <c r="E49" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6669,7 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -6495,6 +6680,11 @@
       <c r="E50" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6701,7 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -6522,6 +6712,11 @@
       <c r="E51" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>teórico</t>
         </is>
       </c>
     </row>
@@ -6538,7 +6733,7 @@
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
@@ -6549,6 +6744,11 @@
       <c r="E52" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>teórico</t>
         </is>
       </c>
     </row>
@@ -6565,7 +6765,7 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
@@ -6576,6 +6776,11 @@
       <c r="E53" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>teórico</t>
         </is>
       </c>
     </row>
@@ -6592,7 +6797,7 @@
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
@@ -6603,6 +6808,11 @@
       <c r="E54" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>teórico</t>
         </is>
       </c>
     </row>
@@ -6619,7 +6829,7 @@
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Teoría e historia de la arquitectura y el diseño</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
@@ -6630,6 +6840,11 @@
       <c r="E55" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>teórico</t>
         </is>
       </c>
     </row>
@@ -6646,7 +6861,7 @@
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Oficio, tecnologías y aprendizaje proyectual</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
@@ -6657,6 +6872,11 @@
       <c r="E56" s="8" t="inlineStr">
         <is>
           <t>nueva</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>teórico</t>
         </is>
       </c>
     </row>
@@ -6673,7 +6893,7 @@
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Personas, interacción y sistemas inclusivos</t>
+          <t>Formación, oficio y teoría del proyecto</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
@@ -6684,6 +6904,11 @@
       <c r="E57" s="8" t="inlineStr">
         <is>
           <t>nueva — separa IA aplicada al diseño democrático/inclusivo de fabricación digital</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>proyectual</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Visualización: leyenda y definición de las dos líneas, proyectos en el panel
- Barra lateral de las tres superficies: leyenda de Fundamentos disciplinares
  y Prácticas proyectuales con modo de investigar, definición breve y cifras
  (sublíneas, proyectos), clicable; nota de polos teórico/proyectual.
- Nodos-línea rotulados siempre en el grafo; tooltip con la definición.
- Panel de detalle: definición de la línea; proyectos 2014-2026 por línea,
  sublínea e investigador (xlsx-loader lee 19_Proyectos).
- Planilla: columnas modo y bajada en 01_Lineas; sello actualizado a los
  nombres nuevos; limpieza de notas LIN-04, 00_Lectura y 15_Decisiones.
- Specs, roadmap y README al régimen de dos líneas; capturas regeneradas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018wL5DZXTvkgua4PoB5SQcj
</commit_message>
<xml_diff>
--- a/mad-map-data-v2.xlsx
+++ b/mad-map-data-v2.xlsx
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="24" min="1" max="1"/>
@@ -657,6 +657,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="16" customHeight="1" s="24">
       <c r="A4" s="26" t="inlineStr">
         <is>
@@ -672,19 +673,19 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Estructura superior. Lo que la Escuela declara y sostiene. BORRADOR.</t>
+          <t>Estructura superior: Fundamentos disciplinares (acerca del proyecto) y Prácticas proyectuales (a través del proyecto), cada una con polo teórico y polo proyectual.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Sublínea (~30)</t>
+          <t>Sublínea (53)</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Pertenece a UNA sola Línea. Granularidad operativa. Banco depurado.</t>
+          <t>Pertenece a UNA sola Línea y a un polo (teórico o proyectual). Granularidad operativa.</t>
         </is>
       </c>
     </row>
@@ -760,80 +761,93 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="16" customHeight="1" s="24">
-      <c r="A14" s="26" t="inlineStr">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Proyecto de investigación o creación 2014-2026 (hoja 19_Proyectos). Pertenece a una Sublínea; participan uno o más Investigadores. La productividad por profesor está en 20_Productividad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Convenciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>BORRADOR (fondo amarillo)</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Filas/celdas con valores propuestos por revisar. La Línea-04 y los mapeos m:n están sujetos a curaduría.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>IDs</t>
+          <t>BORRADOR (fondo amarillo)</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>LIN-NN, SUB-NN, TEM-NNN, INV-NN, LAB-XXX, MOD-NN, SAL-XXX. Estables — no renombrar tras enlazar.</t>
+          <t>Filas o celdas con valores propuestos por revisar. Los mapeos m:n y la asignación de proyectos a sublíneas (19_Proyectos) están sujetos a curaduría.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Cardinalidad Sublínea→Línea</t>
+          <t>IDs</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>1:N estricta (una Sublínea pertenece a UNA Línea). Cambia el linea_id si el ajuste lo amerita.</t>
+          <t>LIN-NN, SUB-NN, TEM-NNN, INV-NN, LAB-XXX, MOD-NN, SAL-XXX. Estables — no renombrar tras enlazar.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Cardinalidad Tema→Sublínea</t>
+          <t>Cardinalidad Sublínea→Línea</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>M:N (un Tema puede colgar de varias Sublíneas). Editar en la hoja 08_Temas (cada fila atribuye un tema a una sublínea y un investigador).</t>
+          <t>1:N estricta (una Sublínea pertenece a UNA Línea). Cambia el linea_id si el ajuste lo amerita.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Cardinalidad Lab→Línea</t>
+          <t>Cardinalidad Tema→Sublínea</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>M:N. Un Lab puede sostener varias Líneas. Editar en 10_Lab_Linea.</t>
+          <t>M:N (un Tema puede colgar de varias Sublíneas). Editar en la hoja 08_Temas (cada fila atribuye un tema a una sublínea y un investigador).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>Cardinalidad Lab→Línea</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>M:N. Un Lab puede sostener varias Líneas. Editar en 10_Lab_Linea.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>Decisiones pendientes</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Hoja 15_Decisiones — preguntas abiertas que afectan el modelo.</t>
         </is>
@@ -2270,7 +2284,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>¿3 o 4 Líneas troncales?</t>
+          <t>¿Cuántas líneas de investigación?</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -2341,7 +2355,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Asignada provisoriamente a LIN-02. Tiene respaldo también en LIN-03. Decidir hogar.</t>
+          <t>Asignada a Prácticas proyectuales (polo proyectual). Tiene respaldo también en Fundamentos disciplinares por el acervo de las travesías. Decidir si queda como puente entre líneas.</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -2363,7 +2377,7 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Asignada provisoriamente a LIN-02 (ecologías). Podría leerse en LIN-01 (inclusión) o quedar transversal.</t>
+          <t>Asignada a Prácticas proyectuales (polo teórico). Podría leerse también en Fundamentos disciplinares (diseño decolonial) o quedar transversal.</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -2779,6 +2793,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -2807,7 +2822,7 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>El doctorado forma investigadores para quienes la obra es origen y prueba de la tesis. Esa obra, sea edificada, fabricada, escrita o dibujada, vale como argumento por sí misma, y el discurso doctoral se construye para hacerla legible y discutible. La pregunta que esa obra está llamada a argumentar es la que el programa hace suya: cómo reinventar el habitar humano, y la responde desde el habitar poético que funda a la Escuela. Las dos líneas del doctorado investigan ese habitar en arquitectura y en diseño: una investiga acerca del proyecto, su formación, su oficio y su teoría; la otra investiga a través del proyecto, sobre la ciudad, el territorio y sus ecologías. Cada línea lleva dentro su contraparte, teórica o proyectual. Doctorarse aquí es haber producido una obra capaz de sostener esos principios al ponerse a prueba y, en su mejor versión, capaz de reformularlos.</t>
+          <t>El doctorado forma investigadores para quienes la obra es origen y prueba de la tesis. Esa obra, sea edificada, fabricada, escrita o dibujada, vale como argumento por sí misma, y el discurso doctoral se construye para hacerla legible y discutible. La pregunta que esa obra está llamada a argumentar es la que el programa hace suya: cómo reinventar el habitar humano, y la responde desde el habitar poético que funda a la Escuela. Las dos líneas del doctorado investigan ese habitar en arquitectura y en diseño: Fundamentos disciplinares investiga acerca del proyecto, lo que sostiene a la disciplina y cómo se transmite; Prácticas proyectuales investiga a través del proyecto, como obra nueva que se inscribe en un contexto y lo modifica. Cada línea lleva dentro su contraparte, teórica o proyectual. Doctorarse aquí es haber producido una obra capaz de sostener esos principios al ponerse a prueba y, en su mejor versión, capaz de reformularlos.</t>
         </is>
       </c>
     </row>
@@ -12831,26 +12846,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="24" min="1" max="1"/>
     <col width="55" customWidth="1" style="24" min="2" max="2"/>
     <col width="95" customWidth="1" style="24" min="3" max="3"/>
     <col width="26" customWidth="1" style="24" min="4" max="4"/>
+    <col width="60" customWidth="1" style="24" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1" s="24">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>01 · Líneas de investigación (2, propuesta septiembre 2026)</t>
+          <t>01 · Líneas de investigación (2, nombres adoptados en octubre de 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>Cada Sublínea pertenece a una Línea y a un polo (teórico | proyectual). Los Laboratorios pueden sostener una o varias Líneas.</t>
+          <t>Dos líneas simétricas, cada una con polo teórico y polo proyectual. Cada Sublínea pertenece a una Línea y a un polo. 'bajada' es la definición breve que muestra la visualización; 'descripción' es el alcance completo.</t>
         </is>
       </c>
     </row>
@@ -12875,6 +12891,16 @@
           <t>estado</t>
         </is>
       </c>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>modo</t>
+        </is>
+      </c>
+      <c r="F4" s="30" t="inlineStr">
+        <is>
+          <t>bajada</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="45" customHeight="1" s="24">
       <c r="A5" s="8" t="inlineStr">
@@ -12897,6 +12923,16 @@
           <t>nombre adoptado 29 sep 2026</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Investigación acerca del proyecto</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Lo que sostiene a la disciplina (su historia, su teoría, su filosofía y sus métodos) y cómo se domina y se transmite en la formación.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="45" customHeight="1" s="24">
       <c r="A6" s="8" t="inlineStr">
@@ -12917,6 +12953,16 @@
       <c r="D6" s="8" t="inlineStr">
         <is>
           <t>nombre adoptado 6 oct 2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Investigación a través del proyecto</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Obra nueva (un edificio, un espacio público, un objeto, un servicio, un sistema) que se inscribe en un contexto y lo modifica.</t>
         </is>
       </c>
     </row>

</xml_diff>